<commit_message>
refactor: organize and fine-tune UI and API automation code
</commit_message>
<xml_diff>
--- a/src/thingsboard_automation/documentation/bug_report.xlsx
+++ b/src/thingsboard_automation/documentation/bug_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abhilashbabu/Documents/ABB/thingsboard-automation/src/thingsboard_automation/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB5BB8D5-7245-2D48-9669-94B772B1E718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26833851-71F6-A947-83FB-C291CE596A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="24960" windowHeight="17220" xr2:uid="{402D9C87-32C1-934B-B37C-CB8746F20C4E}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{402D9C87-32C1-934B-B37C-CB8746F20C4E}"/>
   </bookViews>
   <sheets>
     <sheet name="bugreport" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Bug ID</t>
   </si>
@@ -83,70 +83,43 @@
     <t>BUG-001</t>
   </si>
   <si>
-    <t>Dashboard</t>
-  </si>
-  <si>
-    <t>Telemetry data appears stale</t>
-  </si>
-  <si>
-    <t>Dashboard continues showing the last telemetry value after updates stop</t>
-  </si>
-  <si>
-    <t>User logged in and dashboard opened</t>
-  </si>
-  <si>
-    <t>1. Open dashboard 2. Observe telemetry 3. Stop/wait for telemetry 4. Observe widget</t>
-  </si>
-  <si>
-    <t>Dashboard should indicate that telemetry is stale/offline</t>
-  </si>
-  <si>
-    <t>Last value continues to be displayed without clear stale indication</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
-    <t>demo.thingsboard.io / Chrome / macOS</t>
-  </si>
-  <si>
-    <t>evidence/ui/bug_001.png</t>
-  </si>
-  <si>
     <t>Open</t>
   </si>
   <si>
-    <t>BUG-002</t>
-  </si>
-  <si>
-    <t>Dashboard UI</t>
-  </si>
-  <si>
-    <t>No clear indication of telemetry refresh status</t>
-  </si>
-  <si>
-    <t>User cannot easily determine when the widget was last updated</t>
-  </si>
-  <si>
-    <t>Dashboard loaded</t>
-  </si>
-  <si>
-    <t>1. Open dashboard 2. Observe telemetry widgets 3. Monitor updates</t>
-  </si>
-  <si>
-    <t>Widget should provide clear indication of latest update/freshness</t>
-  </si>
-  <si>
-    <t>No obvious visual indication of last update time on the widget</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>evidence/ui/bug_002.png</t>
+    <t>Authentication / Login</t>
+  </si>
+  <si>
+    <t>Unable to log in to ThingsBoard Demo using the credentials provided in the assignment</t>
+  </si>
+  <si>
+    <t>The user is unable to log in to the ThingsBoard Demo application using the credentials provided for the assignment. The application displays an "Invalid username or password" error, preventing access to the dashboard and blocking further UI validation.</t>
+  </si>
+  <si>
+    <t>User has access to the ThingsBoard Demo login page and uses the credentials provided in the assignment.</t>
+  </si>
+  <si>
+    <t>1. Navigate to `https://demo.thingsboard.io/login`.
+2. Enter username: `tenant@thingsboard.org`
+3. Enter password: `tenant`.
+4. Click  Login.</t>
+  </si>
+  <si>
+    <t>User should successfully authenticate and be redirected to the ThingsBoard dashboard.</t>
+  </si>
+  <si>
+    <t>Login fails and displays the error message "Invalid username or password". The user cannot access the dashboard.</t>
+  </si>
+  <si>
+    <t>Blocker</t>
+  </si>
+  <si>
+    <t>ThingsBoard Demo / Chrome / macOS</t>
+  </si>
+  <si>
+    <t>evidence/ui/login_error.png</t>
   </si>
 </sst>
 </file>
@@ -196,10 +169,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,6 +512,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{642D8B10-5A78-294C-A35F-9E1C79CB28E6}">
   <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="70.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="43.83203125" customWidth="1"/>
+    <col min="11" max="11" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -578,87 +565,49 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="69" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
         <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" t="s">
-        <v>25</v>
-      </c>
+      <c r="L3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>